<commit_message>
NTIS Intraday v1.3 stable baseline with historical datasets
</commit_message>
<xml_diff>
--- a/Intraday/Output/2026-07-22/intraday_backtest_results.xlsx
+++ b/Intraday/Output/2026-07-22/intraday_backtest_results.xlsx
@@ -502,7 +502,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -560,7 +560,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -618,7 +618,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -676,7 +676,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -734,7 +734,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -792,7 +792,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -850,7 +850,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -908,7 +908,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -966,7 +966,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1024,7 +1024,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1082,7 +1082,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1140,7 +1140,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1256,7 +1256,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1314,7 +1314,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1372,7 +1372,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1430,7 +1430,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1488,7 +1488,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1546,7 +1546,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1604,7 +1604,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1662,7 +1662,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1720,7 +1720,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1778,7 +1778,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1836,7 +1836,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1894,7 +1894,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1952,7 +1952,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2010,7 +2010,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2068,7 +2068,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2126,7 +2126,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2184,7 +2184,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2242,7 +2242,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2300,7 +2300,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2358,7 +2358,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2416,7 +2416,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2474,7 +2474,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2532,7 +2532,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2590,7 +2590,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2648,7 +2648,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2764,7 +2764,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2822,7 +2822,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2880,7 +2880,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2938,7 +2938,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2996,7 +2996,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3054,7 +3054,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3112,7 +3112,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3170,7 +3170,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3228,7 +3228,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3286,7 +3286,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3344,7 +3344,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3402,7 +3402,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3460,7 +3460,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3518,7 +3518,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3576,7 +3576,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3634,7 +3634,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3692,7 +3692,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3750,7 +3750,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3808,7 +3808,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3866,7 +3866,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3924,7 +3924,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3982,7 +3982,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -4040,7 +4040,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -4098,7 +4098,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -4156,7 +4156,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -4214,7 +4214,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -4272,7 +4272,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -4330,7 +4330,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -4388,7 +4388,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -4446,7 +4446,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -4504,7 +4504,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -4562,7 +4562,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -4620,7 +4620,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -4678,7 +4678,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -4736,7 +4736,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -4794,7 +4794,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4852,7 +4852,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4910,7 +4910,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4968,7 +4968,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -5026,7 +5026,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -5084,7 +5084,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -5142,7 +5142,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -5200,7 +5200,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -5258,7 +5258,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -5316,7 +5316,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -5374,7 +5374,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -5432,7 +5432,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -5490,7 +5490,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -5548,7 +5548,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -5606,7 +5606,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -5664,7 +5664,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -5722,7 +5722,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -5780,7 +5780,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -5838,7 +5838,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -5896,7 +5896,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -5954,7 +5954,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -6012,7 +6012,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -6070,7 +6070,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -6128,7 +6128,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -6186,7 +6186,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -6244,7 +6244,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -6302,7 +6302,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -6360,7 +6360,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -6418,7 +6418,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -6476,7 +6476,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -6534,7 +6534,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -6592,7 +6592,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -6650,7 +6650,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -6708,7 +6708,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -6766,7 +6766,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -6824,7 +6824,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -6882,7 +6882,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -6940,7 +6940,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -6998,7 +6998,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -7056,7 +7056,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -7114,7 +7114,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -7172,7 +7172,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -7230,7 +7230,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -7288,7 +7288,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -7346,7 +7346,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -7404,7 +7404,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -7462,7 +7462,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -7520,7 +7520,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -7578,7 +7578,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -7636,7 +7636,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -7694,7 +7694,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -7752,7 +7752,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -7810,7 +7810,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -7868,7 +7868,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -7926,7 +7926,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -7984,7 +7984,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -8042,7 +8042,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -8100,7 +8100,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -8158,7 +8158,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -8216,7 +8216,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -8274,7 +8274,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -8332,7 +8332,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -8390,7 +8390,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -8448,7 +8448,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -8506,7 +8506,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -8564,7 +8564,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -8622,7 +8622,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -8680,7 +8680,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -8738,7 +8738,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -8796,7 +8796,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -8854,7 +8854,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -8912,7 +8912,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -8970,7 +8970,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -9028,7 +9028,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -9086,7 +9086,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -9144,7 +9144,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -9202,7 +9202,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -9260,7 +9260,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -9318,7 +9318,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -9376,7 +9376,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -9434,7 +9434,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -9492,7 +9492,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -9550,7 +9550,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -9608,7 +9608,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -9666,7 +9666,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -9724,7 +9724,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -9782,7 +9782,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -9840,7 +9840,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -9898,7 +9898,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -9956,7 +9956,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -10014,7 +10014,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -10072,7 +10072,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -10130,7 +10130,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -10188,7 +10188,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -10246,7 +10246,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -10304,7 +10304,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -10362,7 +10362,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -10420,7 +10420,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -10478,7 +10478,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -10536,7 +10536,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -10594,7 +10594,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -10652,7 +10652,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -10710,7 +10710,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -10768,7 +10768,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -10826,7 +10826,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -10884,7 +10884,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -10942,7 +10942,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -11000,7 +11000,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -11058,7 +11058,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -11116,7 +11116,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -11174,7 +11174,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -11232,7 +11232,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -11290,7 +11290,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -11348,7 +11348,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -11406,7 +11406,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -11464,7 +11464,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -11522,7 +11522,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -11580,7 +11580,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -11638,7 +11638,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -11696,7 +11696,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -11754,7 +11754,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -11812,7 +11812,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -11870,7 +11870,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -11928,7 +11928,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -11986,7 +11986,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -12044,7 +12044,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -12102,7 +12102,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -12160,7 +12160,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -12218,7 +12218,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -12276,7 +12276,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -12334,7 +12334,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -12392,7 +12392,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -12450,7 +12450,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -12508,7 +12508,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -12566,7 +12566,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -12624,7 +12624,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -12682,7 +12682,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -12740,7 +12740,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -12798,7 +12798,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -12856,7 +12856,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -12914,7 +12914,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -12972,7 +12972,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -13030,7 +13030,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -13088,7 +13088,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">

</xml_diff>